<commit_message>
Automate TC_USF_002: searching a non-existent username shows no records, and sync docs
</commit_message>
<xml_diff>
--- a/docs/OrangeHRM-Test-Suite.xlsx
+++ b/docs/OrangeHRM-Test-Suite.xlsx
@@ -722,22 +722,17 @@
   <si>
     <t xml:space="preserve">1. Log in, go to Admin &gt; User Management
 2. Enter a generated username that no user has
-3. Click Search</t>
-  </si>
-  <si>
-    <t>A generated username (qar_ + random) that does not exist</t>
-  </si>
-  <si>
-    <t>The list reports "No Records Found" and shows no row for that username.</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>tests/SearchUserTest.spec.ts (planned)</t>
-  </si>
-  <si>
-    <t>Planned, not automated yet. Creates no data. Seen live: the message appears twice (an info toast and the table text), so the locator must not be strict. Partly exercised already by the not-created checks in TC_UCF_004/005/007, but not as the subject of a test.</t>
+3. Click Search
+4. Check the table's message, the records count text and the table rows</t>
+  </si>
+  <si>
+    <t>A generated username (qar_ + random) that is only generated, never saved, so no user can have it</t>
+  </si>
+  <si>
+    <t>The table shows "No Records Found", the "(N) Records Found" count text is gone, and no data row is left (only the table's header row).</t>
+  </si>
+  <si>
+    <t>Creates no data, so nothing to clean up. Verified live before automating: the words "No Records Found" appear twice - as the table's own &lt;span&gt; and as a fading info toast &lt;p&gt; - so the test asserts on the table's message (filtered by tag), not the toast; the count text disappears; only the header row remains; the search box keeps the typed value. Also observed, NOT asserted: searching "Admi" (part of the existing "Admin") finds nothing - the username search is an exact match, not "starts with". The number of users is never checked: it was 33, then 27, then 4 on different days. Partly exercised before by the not-created checks in TC_UCF_004/005/007, but not as the subject of a test.</t>
   </si>
   <si>
     <t>TC_USF_003</t>
@@ -758,6 +753,12 @@
   </si>
   <si>
     <t>The user is found with the matching role and status filters and not found with Status = Disabled.</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>tests/SearchUserTest.spec.ts (planned)</t>
   </si>
   <si>
     <t>Planned, not automated yet. To verify live: the list's User Role and Status dropdowns (found by label like the Add User form's) and how they combine with the username box.</t>
@@ -2563,18 +2564,18 @@
         <v>205</v>
       </c>
       <c r="I32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="K32" s="4" t="s">
         <v>206</v>
-      </c>
-      <c r="J32" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="K32" s="4" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="33" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>23</v>
@@ -2586,22 +2587,22 @@
         <v>194</v>
       </c>
       <c r="E33" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="G33" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="H33" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="I33" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="H33" s="4" t="s">
+      <c r="J33" s="4" t="s">
         <v>213</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="J33" s="4" t="s">
-        <v>207</v>
       </c>
       <c r="K33" s="4" t="s">
         <v>214</v>
@@ -2633,7 +2634,7 @@
         <v>220</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>221</v>
@@ -2668,7 +2669,7 @@
         <v>227</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J35" s="4" t="s">
         <v>221</v>
@@ -2703,7 +2704,7 @@
         <v>233</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J36" s="4" t="s">
         <v>234</v>
@@ -2738,7 +2739,7 @@
         <v>239</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J37" s="4" t="s">
         <v>234</v>
@@ -2773,7 +2774,7 @@
         <v>245</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J38" s="4" t="s">
         <v>246</v>
@@ -2808,7 +2809,7 @@
         <v>251</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J39" s="4" t="s">
         <v>246</v>
@@ -2843,7 +2844,7 @@
         <v>257</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="J40" s="4" t="s">
         <v>246</v>
@@ -3096,7 +3097,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Automate TC_USF_003: User Role and Status filters narrow the user search, and sync docs
</commit_message>
<xml_diff>
--- a/docs/OrangeHRM-Test-Suite.xlsx
+++ b/docs/OrangeHRM-Test-Suite.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="265">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -743,25 +743,19 @@
   <si>
     <t xml:space="preserve">1. Create an employee and an ESS / Enabled user through the API
 2. Log in, go to Admin &gt; User Management
-3. Search the username with User Role = ESS and Status = Enabled
-4. Check the user is listed
-5. Search the same username with Status = Disabled
-6. Check no records are found</t>
-  </si>
-  <si>
-    <t>Self-created ESS / Enabled user; filters ESS, Enabled, then Disabled</t>
-  </si>
-  <si>
-    <t>The user is found with the matching role and status filters and not found with Status = Disabled.</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>tests/SearchUserTest.spec.ts (planned)</t>
-  </si>
-  <si>
-    <t>Planned, not automated yet. To verify live: the list's User Role and Status dropdowns (found by label like the Add User form's) and how they combine with the username box.</t>
+3. Search the username with User Role = ESS and Status = Enabled; check the user is listed
+4. Search the same username with Status = Disabled; check no records are found
+5. Search again with ESS and Enabled; check the user is listed again
+6. Search the same username with User Role = Admin; check no records are found</t>
+  </si>
+  <si>
+    <t>Self-created ESS / Enabled user; the same username searched with ESS+Enabled, ESS+Disabled, ESS+Enabled, Admin+Enabled</t>
+  </si>
+  <si>
+    <t>The user is found with its own role and status, and NOT found when the Status filter is Disabled or when the User Role filter is Admin. Putting the matching filters back finds the user again. Each "none" shows the table's "No Records Found" with no row.</t>
+  </si>
+  <si>
+    <t>The employee and user are created through the API and deleted by teardown. Verified live before automating: the list's User Role dropdown offers Admin / ESS and Status offers Enabled / Disabled (both found by label with the same helpers as the Add User form); with the username they narrow the result exactly as above; a dropdown keeps its last value between searches, so every search sets both; Reset clears the dropdowns too. The order alternates found / none / found / none ON PURPOSE: shown by mutation that two "none" results in a row, with the second search skipped, PASS WRONGLY on the previous result's message still being on screen. Only filters combined with the username are tested; a role or status filter alone is not (it returns other people's users, whose number changes).</t>
   </si>
   <si>
     <t>TC_UEF_001</t>
@@ -785,6 +779,9 @@
   </si>
   <si>
     <t>The success toast appears and the list shows the user with Status Disabled (other columns unchanged).</t>
+  </si>
+  <si>
+    <t>Planned</t>
   </si>
   <si>
     <t>tests/EditUserTest.spec.ts (planned)</t>
@@ -2599,18 +2596,18 @@
         <v>211</v>
       </c>
       <c r="I33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="K33" s="4" t="s">
         <v>212</v>
-      </c>
-      <c r="J33" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="K33" s="4" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="34" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>12</v>
@@ -2619,33 +2616,33 @@
         <v>32</v>
       </c>
       <c r="D34" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="F34" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E34" s="4" t="s">
+      <c r="G34" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="H34" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="I34" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="H34" s="4" t="s">
+      <c r="J34" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="I34" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J34" s="4" t="s">
+      <c r="K34" s="4" t="s">
         <v>221</v>
-      </c>
-      <c r="K34" s="4" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="35" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>23</v>
@@ -2654,33 +2651,33 @@
         <v>52</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E35" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="G35" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="H35" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="I35" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="K35" s="4" t="s">
         <v>227</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J35" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="36" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>12</v>
@@ -2689,33 +2686,33 @@
         <v>32</v>
       </c>
       <c r="D36" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E36" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="F36" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="G36" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="H36" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="I36" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="H36" s="4" t="s">
+      <c r="J36" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="I36" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J36" s="4" t="s">
+      <c r="K36" s="4" t="s">
         <v>234</v>
-      </c>
-      <c r="K36" s="4" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="37" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>23</v>
@@ -2724,33 +2721,33 @@
         <v>32</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E37" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="F37" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="G37" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="H37" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="I37" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="H37" s="4" t="s">
+      <c r="J37" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="K37" s="4" t="s">
         <v>239</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J37" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="K37" s="4" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="38" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>12</v>
@@ -2762,30 +2759,30 @@
         <v>14</v>
       </c>
       <c r="E38" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="F38" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="G38" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="H38" s="4" t="s">
         <v>244</v>
       </c>
-      <c r="H38" s="4" t="s">
+      <c r="I38" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="J38" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="I38" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J38" s="4" t="s">
+      <c r="K38" s="4" t="s">
         <v>246</v>
-      </c>
-      <c r="K38" s="4" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="39" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>23</v>
@@ -2797,30 +2794,30 @@
         <v>14</v>
       </c>
       <c r="E39" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F39" s="4" t="s">
         <v>249</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>250</v>
       </c>
       <c r="G39" s="4" t="s">
         <v>60</v>
       </c>
       <c r="H39" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="K39" s="4" t="s">
         <v>251</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J39" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="K39" s="4" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="40" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>23</v>
@@ -2832,25 +2829,25 @@
         <v>14</v>
       </c>
       <c r="E40" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="F40" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="G40" s="4" t="s">
         <v>255</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="H40" s="4" t="s">
         <v>256</v>
       </c>
-      <c r="H40" s="4" t="s">
+      <c r="I40" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="K40" s="4" t="s">
         <v>257</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="J40" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="K40" s="4" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="41" spans="9:9" x14ac:dyDescent="0.25"/>
@@ -3047,12 +3044,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B3" s="10">
         <f>COUNTA('OrangeHRM Test Suite'!$A$2:$A$200)</f>
@@ -3072,7 +3069,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B5" s="10">
         <f>COUNTIF('OrangeHRM Test Suite'!$I$2:$I$200,"Planned")</f>
@@ -3088,16 +3085,16 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="B7" s="11" t="s">
         <v>262</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>263</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3172,7 +3169,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B13" s="11">
         <f>SUM(B8:B12)</f>
@@ -3186,7 +3183,7 @@
     </row>
     <row r="15" ht="60" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>

</xml_diff>

<commit_message>
Automate TC_UEF_001: edit a user's status from Enabled to Disabled via the row's edit icon, and sync docs
</commit_message>
<xml_diff>
--- a/docs/OrangeHRM-Test-Suite.xlsx
+++ b/docs/OrangeHRM-Test-Suite.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="267">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -768,26 +768,24 @@
   </si>
   <si>
     <t xml:space="preserve">1. Create an employee and an ESS / Enabled user through the API
-2. Log in, go to Admin &gt; User Management and search the username
+2. Log in, go to Admin &gt; User Management and search the username; check it starts as ESS / Enabled
 3. Click the row's edit (pencil) button
-4. Change Status to Disabled and click Save
-5. Check the success toast
-6. Search the username again and check the row shows Disabled</t>
-  </si>
-  <si>
-    <t>Self-created ESS / Enabled user</t>
-  </si>
-  <si>
-    <t>The success toast appears and the list shows the user with Status Disabled (other columns unchanged).</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>tests/EditUserTest.spec.ts (planned)</t>
-  </si>
-  <si>
-    <t>Planned, not automated yet. To verify live: the edit form's fields, which are locked, the toast text, and whether saving needs the password. Seen live: the row's edit and delete icons are buttons with NO accessible name (only icon classes bi-pencil-fill / bi-trash), so they need an icon-based locator with a comment.</t>
+4. Wait for the edit form to load the user's values (ESS, Enabled, the username)
+5. Change Status to Disabled and click Save
+6. Check the toast "Successfully Updated"
+7. Search the username again and check the row shows Disabled with everything else unchanged</t>
+  </si>
+  <si>
+    <t>Self-created ESS / Enabled user (generated username)</t>
+  </si>
+  <si>
+    <t>The toast "Successfully Updated" appears, the page returns to the user list, and searching the username shows exactly one row: same username, ESS, same employee name, and Status Disabled.</t>
+  </si>
+  <si>
+    <t>tests/EditUserTest.spec.ts</t>
+  </si>
+  <si>
+    <t>The employee and user are created through the API and deleted by teardown (which removes the user). Verified live before automating: the row's edit and delete icons are buttons with NO accessible name (bare icons), so the edit button is found by its icon class bi-pencil-fill inside the row, with a comment; the edit form lives at /admin/saveSystemUser/&lt;id&gt; with the heading "Edit User"; it OPENS EMPTY and fills in about 3 seconds later, so the test waits for the username to appear before touching anything (a change made earlier could be overwritten or saved against blank fields); "Change Password ?" is unchecked, so no password is needed; Save sends one PUT /api/v2/admin/users/&lt;id&gt; and the toast shows BEFORE the redirect, which lands a few seconds later; the form shows the employee name with a doubled space where the list has one, so the name is only checked in the list. Shown by mutation: the "Successfully Updated" toast also appears when NOTHING was changed, so the toast does not prove the edit - the final list row does. Only ESS and Enabled -&gt; Disabled is covered; changing the role is not (that could create an Admin on the shared demo).</t>
   </si>
   <si>
     <t>TC_UEF_002</t>
@@ -806,6 +804,12 @@
   </si>
   <si>
     <t>Username shows "Already exists" (as on the Add User form), the page stays on the edit form, and the second user keeps its original username.</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>tests/EditUserTest.spec.ts (planned)</t>
   </si>
   <si>
     <t>Planned, not automated yet. To verify live whether the edit form checks uniqueness the same way as the Add User form ("Already exists" appeared as soon as the value was typed there).</t>
@@ -825,6 +829,9 @@
 3. Click the row's delete (trash) button
 4. Confirm the deletion in the dialog
 5. Search the username again</t>
+  </si>
+  <si>
+    <t>Self-created ESS / Enabled user</t>
   </si>
   <si>
     <t>A success toast appears and searching the username then returns "No Records Found". The employee still exists (only the user is deleted).</t>
@@ -2631,18 +2638,18 @@
         <v>218</v>
       </c>
       <c r="I34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J34" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="J34" s="4" t="s">
+      <c r="K34" s="4" t="s">
         <v>220</v>
-      </c>
-      <c r="K34" s="4" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="35" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>23</v>
@@ -2654,30 +2661,30 @@
         <v>214</v>
       </c>
       <c r="E35" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="G35" s="4" t="s">
         <v>224</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="H35" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="H35" s="4" t="s">
+      <c r="I35" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>219</v>
-      </c>
       <c r="J35" s="4" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="K35" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>12</v>
@@ -2686,33 +2693,33 @@
         <v>32</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K36" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="37" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>23</v>
@@ -2721,33 +2728,33 @@
         <v>32</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="K37" s="4" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>12</v>
@@ -2759,30 +2766,30 @@
         <v>14</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="39" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>23</v>
@@ -2794,30 +2801,30 @@
         <v>14</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="G39" s="4" t="s">
         <v>60</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="40" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>23</v>
@@ -2829,25 +2836,25 @@
         <v>14</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="41" spans="9:9" x14ac:dyDescent="0.25"/>
@@ -3044,12 +3051,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B3" s="10">
         <f>COUNTA('OrangeHRM Test Suite'!$A$2:$A$200)</f>
@@ -3069,7 +3076,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B5" s="10">
         <f>COUNTIF('OrangeHRM Test Suite'!$I$2:$I$200,"Planned")</f>
@@ -3085,16 +3092,16 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3169,7 +3176,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B13" s="11">
         <f>SUM(B8:B12)</f>
@@ -3183,7 +3190,7 @@
     </row>
     <row r="15" ht="60" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>

</xml_diff>

<commit_message>
Automate TC_UDF_001: delete a user via the row's delete icon and confirm only the user is removed, and sync docs
</commit_message>
<xml_diff>
--- a/docs/OrangeHRM-Test-Suite.xlsx
+++ b/docs/OrangeHRM-Test-Suite.xlsx
@@ -794,25 +794,24 @@
     <t>Editing A User To A Username That Is Already Taken Is Rejected</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Create two employees and one user each through the API
-2. Log in, search the second user and open its edit form
+    <t xml:space="preserve">1. Create two employees and one ESS / Enabled user each through the API
+2. Log in, search the second user and open its edit form; wait for it to load
 3. Change the username to the first user's username
-4. Click Save</t>
-  </si>
-  <si>
-    <t>Two self-created users with different generated usernames</t>
-  </si>
-  <si>
-    <t>Username shows "Already exists" (as on the Add User form), the page stays on the edit form, and the second user keeps its original username.</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>tests/EditUserTest.spec.ts (planned)</t>
-  </si>
-  <si>
-    <t>Planned, not automated yet. To verify live whether the edit form checks uniqueness the same way as the Add User form ("Already exists" appeared as soon as the value was typed there).</t>
+4. Check only Username shows a message
+5. Click Save
+6. Check the page is still the edit form, the message remains, and no success toast appeared
+7. Click Cancel
+8. Search the second user's ORIGINAL username and check it is unchanged
+9. Search the taken username and check it still shows exactly the first user</t>
+  </si>
+  <si>
+    <t>Two self-created ESS / Enabled users with different generated usernames; the second user's username changed to the first's</t>
+  </si>
+  <si>
+    <t>Username shows "Already exists" and no other field shows an error. Save does not go through: the page stays on /admin/saveSystemUser/&lt;id&gt; with no success toast. After Cancel, the second user is still listed under its original username, and the taken username shows exactly one record - the first user's.</t>
+  </si>
+  <si>
+    <t>Both employees and their users are created through the API and deleted by teardown (which removes the users). Verified live before automating: the edit form checks uniqueness exactly like the Add User form - "Already exists" appears as soon as the username is typed, from the same server check (which also sends the user's own id); typing a user's OWN username again is NOT flagged; Save sends no PUT (only the validation request), shows no toast and stays on the form. Shown by mutation: if the rename did go through, the final "original username" check fails. The last two checks go through assertUserListed, which waits for that username's own row, so they cannot pass on the previous search's "(1) Record Found" still being on screen (a trap hit while probing). Also seen in that mutation: a search made right after a Save redirect did not apply (the list stayed at "(30) Records Found") - the second time this was seen after the TC_UCF_008 flake; this test does not search after a save redirect.</t>
   </si>
   <si>
     <t>TC_UDF_001</t>
@@ -824,23 +823,23 @@
     <t>Delete A User From The List</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Create an employee and a user for it through the API
-2. Log in, go to Admin &gt; User Management and search the username
-3. Click the row's delete (trash) button
-4. Confirm the deletion in the dialog
-5. Search the username again</t>
-  </si>
-  <si>
-    <t>Self-created ESS / Enabled user</t>
-  </si>
-  <si>
-    <t>A success toast appears and searching the username then returns "No Records Found". The employee still exists (only the user is deleted).</t>
-  </si>
-  <si>
-    <t>tests/DeleteUserTest.spec.ts (planned)</t>
-  </si>
-  <si>
-    <t>Planned, not automated yet. Deletes only a user this test created. To verify live: the confirmation dialog's text and buttons (my first probe's dialog locator did not match, so they are not known yet) and the toast text.</t>
+    <t xml:space="preserve">1. Create an employee and an ESS / Enabled user for it through the API
+2. Log in, go to Admin &gt; User Management, search the username and check it is listed
+3. Click the row's delete (trash) button; check the confirmation asks "Are you Sure?"
+4. Click "Yes, Delete"
+5. Check the toast "Successfully Deleted" and that the dialog closed
+6. Check the list no longer shows the user
+7. Search the username again and check no user is found
+8. Check the employee still exists</t>
+  </si>
+  <si>
+    <t>The confirmation ("Are you Sure? The selected record will be permanently deleted...") appears; after "Yes, Delete" the toast "Successfully Deleted" shows and the dialog closes. The list, and a fresh search, report "No Records Found" for that username. The employee still exists - only the user was deleted.</t>
+  </si>
+  <si>
+    <t>tests/DeleteUserTest.spec.ts</t>
+  </si>
+  <si>
+    <t>Deletes only a user this test created. The employee and user are created through the API; the employee is deleted by teardown at the end, so "the employee survives" is checked through the API (TestData.employeeExists, matched on employee number because the id search is a substring match). Verified live before automating: the confirmation is a real role="dialog" with accessible "No, Cancel" and "Yes, Delete" buttons (my first probe's selector was simply wrong); the row's trash button, like the edit button, has no accessible name and is found by its icon class bi-trash; Yes sends one DELETE /api/v2/admin/users with the user ids, shows "Successfully Deleted", stays on the list (NO redirect) and the list refreshes itself, keeping the username filter. Shown by mutation: never confirming, or clicking "No, Cancel", leaves no toast and fails at the toast step; the employee check reads real state. The cancel path (user stays) is the separate planned TC_UDF_002.</t>
   </si>
   <si>
     <t>TC_UDF_002</t>
@@ -855,7 +854,16 @@
 4. Check the dialog closed and the user is still listed</t>
   </si>
   <si>
+    <t>Self-created ESS / Enabled user</t>
+  </si>
+  <si>
     <t>The dialog closes, no success toast appears, and the user is still listed with the same values.</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>tests/DeleteUserTest.spec.ts (planned)</t>
   </si>
   <si>
     <t>Planned, not automated yet. To verify live: the dialog's cancel button name ("No, Cancel" is the expected wording, unconfirmed).</t>
@@ -2673,18 +2681,18 @@
         <v>225</v>
       </c>
       <c r="I35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="K35" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="J35" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="K35" s="4" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="36" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>12</v>
@@ -2693,33 +2701,33 @@
         <v>32</v>
       </c>
       <c r="D36" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="F36" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="E36" s="4" t="s">
+      <c r="G36" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="H36" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="I36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J36" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="K36" s="4" t="s">
         <v>233</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="J36" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="K36" s="4" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="37" ht="78" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>23</v>
@@ -2728,25 +2736,25 @@
         <v>32</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E37" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="H37" s="4" t="s">
         <v>238</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="I37" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="G37" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="H37" s="4" t="s">
+      <c r="J37" s="4" t="s">
         <v>240</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="J37" s="4" t="s">
-        <v>235</v>
       </c>
       <c r="K37" s="4" t="s">
         <v>241</v>
@@ -2778,7 +2786,7 @@
         <v>246</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="J38" s="4" t="s">
         <v>247</v>
@@ -2813,7 +2821,7 @@
         <v>252</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="J39" s="4" t="s">
         <v>247</v>
@@ -2848,7 +2856,7 @@
         <v>258</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="J40" s="4" t="s">
         <v>247</v>
@@ -3101,7 +3109,7 @@
         <v>8</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>